<commit_message>
run(大小周期共振): callback schedules (D030–D035, all on_demand; reversal async), event-driven driver regenerated, S8 re-frozen; stub docstrings show schedule; on_demand event
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workspace/大小周期共振/S6_terms_defined.xlsx
+++ b/workspace/大小周期共振/S6_terms_defined.xlsx
@@ -1308,7 +1308,7 @@
       <c r="O12" s="4" t="inlineStr"/>
       <c r="P12" s="4" t="inlineStr">
         <is>
-          <t>原文强调'判断不是预测而是跟随'，只需知道当下方向，但未给出方向的判定方法（用什么指标/结构）。 S3 D003/D004：“高一级周期出现转向信号”与本判定合并为同一件事（T028 并入）；“顺势”原则由本判定落实（T003 并入）。</t>
+          <t>原文强调'判断不是预测而是跟随'，只需知道当下方向，但未给出方向的判定方法（用什么指标/结构）。 S3 D003/D004：“高一级周期出现转向信号”与本判定合并为同一件事（T028 并入）；“顺势”原则由本判定落实（T003 并入）。 schedule: on_demand/sync（D030：用于开仓的方向判定由下游调用方决定调用频率）。</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       <c r="O14" s="4" t="inlineStr"/>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>原文只说在小周期入场并只执行与大周期同向的信号，未定义入场信号本身；且明确'不要试图找完美入场点'。</t>
+          <t>原文只说在小周期入场并只执行与大周期同向的信号，未定义入场信号本身；且明确'不要试图找完美入场点'。 schedule: on_demand/sync（D031：空仓且大周期方向判定非空（多/空）时反复评估，间隔/频率由下游调用方决定）。</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       <c r="O15" s="4" t="inlineStr"/>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>初始止损按小周期设置、'很近'，但未给出具体位置（结构位/固定点数/波动）；原文只论证为何不用大周期止损。</t>
+          <t>初始止损按小周期设置、'很近'，但未给出具体位置（结构位/固定点数/波动）；原文只论证为何不用大周期止损。 schedule: on_demand/sync（D032：与入场信号同一事件，入场信号为“入场”后立即同步调用一次）。</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       <c r="O21" s="4" t="inlineStr"/>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>持仓期间止损只按大周期信号推进，但'大周期的信号'是什么、推进到哪里未说明；原文亦未明说止损只进不退，但'朝有利方向移动'暗示如此。</t>
+          <t>持仓期间止损只按大周期信号推进，但'大周期的信号'是什么、推进到哪里未说明；原文亦未明说止损只进不退，但'朝有利方向移动'暗示如此。 schedule: on_demand/sync（D034：移损至成本后，由下游调用方决定评估频率）。</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       <c r="O22" s="4" t="inlineStr"/>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>两种出场方式之一，判定方法未定义；与'不主动平仓'并列时略有张力（反转出场是否算主动平仓）。 S3 D001：趋势反转出场是独立于打止损的平仓路径，大周期出现趋势反转即主动清仓。</t>
+          <t>两种出场方式之一，判定方法未定义；与'不主动平仓'并列时略有张力（反转出场是否算主动平仓）。 S3 D001：趋势反转出场是独立于打止损的平仓路径，大周期出现趋势反转即主动清仓。 schedule: on_demand/async（D035：持仓期由下游调用方决定频率，允许异步慢判断，返回 None 沿用上次结果）。</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       <c r="O25" s="4" t="inlineStr"/>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>移损至成本的触发条件；'一定'/'一段'的幅度未量化。 S3 D002：有利运动在大周期上判断（原文说“小周期出现有利运动”，以用户修订为准）。</t>
+          <t>移损至成本的触发条件；'一定'/'一段'的幅度未量化。 S3 D002：有利运动在大周期上判断（原文说“小周期出现有利运动”，以用户修订为准）。 schedule: on_demand/sync（D033：持仓且未移损至成本时，由下游调用方决定评估频率）。</t>
         </is>
       </c>
     </row>

</xml_diff>